<commit_message>
Cap nhat danh muc van ban
</commit_message>
<xml_diff>
--- a/raw/Danh_muc_van_ban_phap_luat.xlsx
+++ b/raw/Danh_muc_van_ban_phap_luat.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh_muc" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong hop" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="144525" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
     <numFmt numFmtId="166" formatCode="_-* #,##0\ &quot;₫&quot;_-;\-* #,##0\ &quot;₫&quot;_-;_-* &quot;-&quot;\ &quot;₫&quot;_-;_-@_-"/>
     <numFmt numFmtId="167" formatCode="_-* #,##0.00\ &quot;₫&quot;_-;\-* #,##0.00\ &quot;₫&quot;_-;_-* &quot;-&quot;??\ &quot;₫&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="29">
     <font>
       <name val="Carlito"/>
       <charset val="134"/>
@@ -205,6 +206,17 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="34">
@@ -661,7 +673,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -692,6 +704,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1072,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col width="6" customWidth="1" style="1" min="1" max="1"/>
@@ -1081,8 +1105,10 @@
     <col width="20" customWidth="1" style="1" min="4" max="4"/>
     <col width="32" customWidth="1" style="1" min="5" max="5"/>
     <col width="65" customWidth="1" style="1" min="6" max="6"/>
-    <col width="50" customWidth="1" style="1" min="7" max="7"/>
-    <col width="40" customWidth="1" style="1" min="8" max="16378"/>
+    <col width="24" customWidth="1" style="1" min="7" max="7"/>
+    <col width="10" customWidth="1" style="1" min="8" max="16378"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1116,14 +1142,24 @@
           <t>Link nguồn / tải / tra cứu</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
-        <is>
-          <t>Đối chiếu với bản gốc (Claude)</t>
-        </is>
-      </c>
-      <c r="H1" s="9" t="inlineStr">
-        <is>
-          <t>Tên trong danh mục cũ (Long ghi)</t>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Định dạng gốc</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Số trang</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Cách lấy chữ</t>
+        </is>
+      </c>
+      <c r="J1" s="9" t="inlineStr">
+        <is>
+          <t>Đối chiếu với bản gốc</t>
         </is>
       </c>
     </row>
@@ -1156,12 +1192,24 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/01/108-qh15.signed.pdf</t>
         </is>
       </c>
-      <c r="G2" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H2" s="11" t="n"/>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="n">
+        <v>65</v>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J2" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="33.6" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -1192,14 +1240,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/7/252-ndcp.signed.pdf</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H3" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định quy định chi tiết và hướng dẫn thi hành Luật Quản lý thuế</t>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="n">
+        <v>133</v>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1232,14 +1288,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/7/255-ndcp.signed.pdf</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H4" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định về quản lý thuế đối với giao dịch liên kết</t>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="n">
+        <v>77</v>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1272,14 +1336,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2020/10/125.signed.pdf</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định về xử phạt vi phạm hành chính về thuế, hóa đơn</t>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>87</v>
+      </c>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1312,14 +1384,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/12/310-cp.signed.pdf</t>
         </is>
       </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định sửa đổi Nghị định 125/2020/NĐ-CP</t>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1352,14 +1432,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/7/291_2026_nd-cp_21072026-signed.signed.pdf</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định sửa đổi quy định xử phạt vi phạm về thuế, hóa đơn</t>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1392,14 +1480,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/7/89-btc.signed.pdf</t>
         </is>
       </c>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư hướng dẫn Luật Quản lý thuế và Nghị định 252/2026/NĐ-CP</t>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>839</v>
+      </c>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1432,12 +1528,24 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/7/90-btc.signed.pdf</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H9" s="11" t="n"/>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>196</v>
+      </c>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -1468,14 +1576,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/7/254-ndcp.signed.pdf</t>
         </is>
       </c>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định về hóa đơn điện tử, chứng từ điện tử</t>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>55</v>
+      </c>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1508,14 +1624,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/7/91-btc.signed.pdf</t>
         </is>
       </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H11" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư hướng dẫn về hóa đơn, chứng từ điện tử</t>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>97</v>
+      </c>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1548,12 +1672,24 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/01/luat48.pdf</t>
         </is>
       </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="n"/>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>PDF có chữ (Công báo)</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>Đọc lớp chữ</t>
+        </is>
+      </c>
+      <c r="J12" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -1584,14 +1720,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/01/luat149.signed.pdf</t>
         </is>
       </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
-          <t>Luật sửa đổi, bổ sung một số điều của Luật Thuế GTGT</t>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1624,14 +1768,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/5/09-qh.signed.pdf</t>
         </is>
       </c>
-      <c r="G14" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>Luật sửa đổi các luật về thuế (bao gồm GTGT, TNCN, TNDN, TTĐB)</t>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J14" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1664,14 +1816,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/7/181nd.signed.pdf</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H15" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định hướng dẫn Luật Thuế GTGT</t>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>75</v>
+      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J15" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1704,14 +1864,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/7/174nd.signed.pdf</t>
         </is>
       </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định về chính sách giảm thuế GTGT</t>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="n">
+        <v>56</v>
+      </c>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1744,14 +1912,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/01/359-nd.signed.pdf</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H17" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định sửa đổi Nghị định 181/2025/NĐ-CP</t>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1784,14 +1960,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/4/144-ndcp.signed.pdf</t>
         </is>
       </c>
-      <c r="G18" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định sửa đổi Nghị định 181/2025/NĐ-CP và 359/2025/NĐ-CP</t>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="n">
+        <v>23</v>
+      </c>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J18" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1824,14 +2008,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/7/69-btc.signed.pdf</t>
         </is>
       </c>
-      <c r="G19" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H19" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư hướng dẫn Luật Thuế GTGT và Nghị định 181/2025/NĐ-CP</t>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1864,14 +2056,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/7/77-btc.pdf</t>
         </is>
       </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư về dịch vụ kinh doanh chứng khoán và chuyển nhượng chứng khoán theo Nghị định 181/2025/NĐ-CP</t>
+      <c r="G20" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -1904,14 +2104,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/01/101-bnnmt.pdf</t>
         </is>
       </c>
-      <c r="G21" s="11" t="inlineStr">
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>PDF convert từ Word</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>Đọc lớp chữ</t>
+        </is>
+      </c>
+      <c r="J21" s="11" t="inlineStr">
         <is>
           <t>Đúng văn bản; số và ngày (31/12/2025) điền tay trên file, file không có trang chữ ký</t>
-        </is>
-      </c>
-      <c r="H21" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư hướng dẫn các loại máy chuyên dùng phục vụ sản xuất nông nghiệp liên quan thuế GTGT</t>
         </is>
       </c>
     </row>
@@ -1944,12 +2152,24 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/01/luat109-2025.pdf</t>
         </is>
       </c>
-      <c r="G22" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H22" s="11" t="n"/>
+      <c r="G22" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J22" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1980,14 +2200,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/7/253m-ndcp.signed.pdf</t>
         </is>
       </c>
-      <c r="G23" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H23" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định hướng dẫn Luật Thuế thu nhập cá nhân</t>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="n">
+        <v>61</v>
+      </c>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2020,14 +2248,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/7/87-btc.signed.pdf</t>
         </is>
       </c>
-      <c r="G24" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H24" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư hướng dẫn Luật Thuế TNCN và Nghị định 253/2026/NĐ-CP</t>
+      <c r="G24" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2060,12 +2296,24 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/7/67qh.signed.pdf</t>
         </is>
       </c>
-      <c r="G25" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H25" s="11" t="n"/>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J25" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -2096,14 +2344,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/12/320-ndcp.signed.pdf</t>
         </is>
       </c>
-      <c r="G26" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H26" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định hướng dẫn Luật Thuế thu nhập doanh nghiệp</t>
+      <c r="G26" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H26" s="13" t="n">
+        <v>76</v>
+      </c>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J26" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2136,14 +2392,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/01/20nd.signed.pdf</t>
         </is>
       </c>
-      <c r="G27" s="11" t="inlineStr">
+      <c r="G27" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="n">
+        <v>23</v>
+      </c>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J27" s="11" t="inlineStr">
         <is>
           <t>Đúng số hiệu thầy giao; nội dung là hướng dẫn Nghị quyết 198/2025/QH15 (có ưu đãi thuế TNDN), không phải hướng dẫn Luật Thuế TNDN</t>
-        </is>
-      </c>
-      <c r="H27" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định số 20/2026/NĐ-CP (cần đối chiếu trích yếu)</t>
         </is>
       </c>
     </row>
@@ -2176,14 +2440,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/4/141-ndcp.signed.pdf</t>
         </is>
       </c>
-      <c r="G28" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H28" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định sửa đổi cả Nghị định 68/2026/NĐ-CP và Nghị định 320/2025/NĐ-CP</t>
+      <c r="G28" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H28" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J28" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2216,14 +2488,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/6/245-ndcp.signed.pdf</t>
         </is>
       </c>
-      <c r="G29" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H29" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định gia hạn thời hạn nộp một số khoản thuế và tiền thuê đất năm 2026</t>
+      <c r="G29" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="I29" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J29" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2256,14 +2536,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/3/20-btc.pdf</t>
         </is>
       </c>
-      <c r="G30" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H30" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư hướng dẫn Luật Thuế TNDN và Nghị định 320/2025/NĐ-CP</t>
+      <c r="G30" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H30" s="13" t="n">
+        <v>22</v>
+      </c>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J30" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2296,14 +2584,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/3/68-ndcp.signed.pdf</t>
         </is>
       </c>
-      <c r="G31" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H31" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định về chính sách thuế và quản lý thuế đối với hộ kinh doanh, cá nhân kinh doanh</t>
+      <c r="G31" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H31" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="I31" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J31" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2336,14 +2632,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/4/141-ndcp.signed.pdf</t>
         </is>
       </c>
-      <c r="G32" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H32" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định 141/2026/NĐ-CP sửa đổi Nghị định 68/2026/NĐ-CP</t>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J32" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2376,14 +2680,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/01/152-btc.pdf</t>
         </is>
       </c>
-      <c r="G33" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H33" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư hướng dẫn kế toán hộ kinh doanh, cá nhân kinh doanh</t>
+      <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J33" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2416,14 +2728,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/3/18-btc.signed.pdf</t>
         </is>
       </c>
-      <c r="G34" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H34" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư về hồ sơ, thủ tục quản lý thuế đối với hộ kinh doanh, cá nhân kinh doanh</t>
+      <c r="G34" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H34" s="13" t="n">
+        <v>44</v>
+      </c>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2456,14 +2776,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/5/50-btc.signed.pdf</t>
         </is>
       </c>
-      <c r="G35" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H35" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư sửa đổi Thông tư 18/2026/TT-BTC</t>
+      <c r="G35" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J35" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2496,12 +2824,24 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2020/07/59.signed.pdf, https://datafiles.chinhphu.vn/cpp/files/vbpq/2020/07/59tiep.pdf</t>
         </is>
       </c>
-      <c r="G36" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H36" s="11" t="n"/>
+      <c r="G36" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H36" s="13" t="n">
+        <v>141</v>
+      </c>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J36" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -2532,14 +2872,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2022/07/03-2022-qh15..pdf</t>
         </is>
       </c>
-      <c r="G37" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H37" s="11" t="inlineStr">
-        <is>
-          <t>Luật sửa đổi nhiều luật, trong đó có Luật Doanh nghiệp</t>
+      <c r="G37" s="13" t="inlineStr">
+        <is>
+          <t>PDF có chữ (Công báo)</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>Đọc lớp chữ</t>
+        </is>
+      </c>
+      <c r="J37" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2572,12 +2920,24 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/7/76qh.signed.pdf</t>
         </is>
       </c>
-      <c r="G38" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H38" s="11" t="n"/>
+      <c r="G38" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H38" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J38" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
@@ -2608,12 +2968,24 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/7/168nd.signed.pdf</t>
         </is>
       </c>
-      <c r="G39" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H39" s="11" t="n"/>
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H39" s="14" t="n">
+        <v>122</v>
+      </c>
+      <c r="I39" s="14" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J39" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="28.8" customHeight="1">
       <c r="A40" s="3" t="n">
@@ -2644,14 +3016,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/7/296_2026_nd-cp_23072026-signed.signed.pdf</t>
         </is>
       </c>
-      <c r="G40" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H40" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định sửa đổi Nghị định 168/2025/NĐ-CP</t>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H40" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="I40" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J40" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2684,14 +3064,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/7/68-btc.pdf</t>
         </is>
       </c>
-      <c r="G41" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H41" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư ban hành biểu mẫu đăng ký doanh nghiệp, đăng ký hộ kinh doanh</t>
+      <c r="G41" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H41" s="13" t="n">
+        <v>266</v>
+      </c>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J41" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2724,14 +3112,22 @@
           <t>https://congbao.chinhphu.vn/van-ban/thong-tu-so-99-2025-tt-btc-46529.htm</t>
         </is>
       </c>
-      <c r="G42" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H42" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư về chế độ kế toán doanh nghiệp</t>
+      <c r="G42" s="14" t="inlineStr">
+        <is>
+          <t>PDF có chữ (Công báo)</t>
+        </is>
+      </c>
+      <c r="H42" s="14" t="n">
+        <v>74</v>
+      </c>
+      <c r="I42" s="14" t="inlineStr">
+        <is>
+          <t>Đọc lớp chữ</t>
+        </is>
+      </c>
+      <c r="J42" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2764,14 +3160,22 @@
           <t>https://congbao.chinhphu.vn/van-ban/thong-tu-so-58-2026-tt-btc-469663.htm</t>
         </is>
       </c>
-      <c r="G43" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H43" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư được mô tả là chế độ kế toán doanh nghiệp siêu nhỏ</t>
+      <c r="G43" s="13" t="inlineStr">
+        <is>
+          <t>PDF convert từ Word</t>
+        </is>
+      </c>
+      <c r="H43" s="13" t="n">
+        <v>33</v>
+      </c>
+      <c r="I43" s="13" t="inlineStr">
+        <is>
+          <t>Đọc lớp chữ</t>
+        </is>
+      </c>
+      <c r="J43" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2804,14 +3208,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/01/152-btc.pdf</t>
         </is>
       </c>
-      <c r="G44" s="11" t="inlineStr">
+      <c r="G44" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H44" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="I44" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J44" s="11" t="inlineStr">
         <is>
           <t>Dùng chung file TT152_2025_BTC.pdf ở nhóm VI (đã xóa bản trùng TT52 đặt sai tên)</t>
-        </is>
-      </c>
-      <c r="H44" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư được mô tả là hướng dẫn kế toán cho hộ kinh doanh, cá nhân kinh doanh</t>
         </is>
       </c>
     </row>
@@ -2844,14 +3256,22 @@
           <t>https://congbao.chinhphu.vn/van-ban/thong-tu-so-71-2024-tt-btc-42903.htm</t>
         </is>
       </c>
-      <c r="G45" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H45" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư được mô tả là chế độ kế toán hợp tác xã</t>
+      <c r="G45" s="13" t="inlineStr">
+        <is>
+          <t>PDF có chữ (Công báo)</t>
+        </is>
+      </c>
+      <c r="H45" s="13" t="n">
+        <v>92</v>
+      </c>
+      <c r="I45" s="13" t="inlineStr">
+        <is>
+          <t>Đọc lớp chữ</t>
+        </is>
+      </c>
+      <c r="J45" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -2884,14 +3304,22 @@
           <t>https://ketoananpha.vn/uploads/files/Van-ban-luat/Ke-toan-Kiem-toan/Thong-tu-133_2016_TT-BTC.doc (bản Word, không phải trang chính thức)</t>
         </is>
       </c>
-      <c r="G46" s="11" t="inlineStr">
+      <c r="G46" s="13" t="inlineStr">
+        <is>
+          <t>Word gốc (.doc)</t>
+        </is>
+      </c>
+      <c r="H46" s="13" t="n">
+        <v>115</v>
+      </c>
+      <c r="I46" s="13" t="inlineStr">
+        <is>
+          <t>Đọc trực tiếp</t>
+        </is>
+      </c>
+      <c r="J46" s="11" t="inlineStr">
         <is>
           <t>Đã bổ sung – bản Word từ ketoananpha.vn (nguồn không chính thức), đã kiểm tra số hiệu và ngày ban hành</t>
-        </is>
-      </c>
-      <c r="H46" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư hướng dẫn chế độ kế toán doanh nghiệp nhỏ và vừa</t>
         </is>
       </c>
     </row>
@@ -2924,12 +3352,24 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2024/9/41-2024-qh15.pdf</t>
         </is>
       </c>
-      <c r="G47" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H47" s="11" t="n"/>
+      <c r="G47" s="13" t="inlineStr">
+        <is>
+          <t>PDF có chữ (Công báo)</t>
+        </is>
+      </c>
+      <c r="H47" s="13" t="n">
+        <v>88</v>
+      </c>
+      <c r="I47" s="13" t="inlineStr">
+        <is>
+          <t>Đọc lớp chữ</t>
+        </is>
+      </c>
+      <c r="J47" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="33.6" customHeight="1">
       <c r="A48" s="3" t="n">
@@ -2960,14 +3400,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/10/274-nd.signed.pdf</t>
         </is>
       </c>
-      <c r="G48" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H48" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định về chậm đóng, trốn đóng BHXH/BHTN và khiếu nại, tố cáo</t>
+      <c r="G48" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H48" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="I48" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J48" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3000,14 +3448,22 @@
           <t>http://datafiles.chinhphu.vn/cpp/files/vbpq/2025/6/158-ndcp.signed.pdf</t>
         </is>
       </c>
-      <c r="G49" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H49" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định hướng dẫn BHXH bắt buộc</t>
+      <c r="G49" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H49" s="13" t="n">
+        <v>52</v>
+      </c>
+      <c r="I49" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J49" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3040,14 +3496,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/6/159-cp.signed.pdf</t>
         </is>
       </c>
-      <c r="G50" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H50" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định hướng dẫn BHXH tự nguyện</t>
+      <c r="G50" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H50" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="I50" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J50" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3080,14 +3544,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/7/176nd.signed.pdf</t>
         </is>
       </c>
-      <c r="G51" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H51" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định về trợ cấp hưu trí xã hội</t>
+      <c r="G51" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H51" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I51" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J51" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3120,14 +3592,22 @@
           <t>https://ebh.vn/Download/vanbanphapquy/thong-tu-12-2025-TT-BNV.pdf</t>
         </is>
       </c>
-      <c r="G52" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H52" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư của Bộ Nội vụ (cần đối chiếu đúng nội dung BHXH trong danh sách)</t>
+      <c r="G52" s="14" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H52" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="I52" s="14" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J52" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3160,14 +3640,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/7/11-bnv.pdf</t>
         </is>
       </c>
-      <c r="G53" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H53" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư của Bộ Nội vụ (cần đối chiếu đúng nội dung BHXH trong danh sách)</t>
+      <c r="G53" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H53" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="I53" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J53" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3200,14 +3688,22 @@
           <t>https://bvtb.org.vn/thong-tu-25-2025-tt-byt-ngay-30-thang-6-nam-2025-quy-dinh-chi-tiet-thi-hanh-luat-bao-hiem-xa-hiem-xa-hoi-luat-an-toan-ve-sinh-lao-dong-ve-linh-vuc-y-te-va-mot-so-dieu-cua-luat-kham-benh-chua-benh/</t>
         </is>
       </c>
-      <c r="G54" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H54" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư của Bộ Y tế (cần đối chiếu đúng nội dung BHXH trong danh sách)</t>
+      <c r="G54" s="14" t="inlineStr">
+        <is>
+          <t>PDF có chữ (Công báo)</t>
+        </is>
+      </c>
+      <c r="H54" s="14" t="n">
+        <v>55</v>
+      </c>
+      <c r="I54" s="14" t="inlineStr">
+        <is>
+          <t>Đọc lớp chữ</t>
+        </is>
+      </c>
+      <c r="J54" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3240,14 +3736,22 @@
           <t>https://vbpl.vn/van-ban/chi-tiet/thong-tu-so-60-2025-tt-byt-quy-dinh-ve-benh-nghe-nghiep-duoc-huong-bao-hiem-xa-hoi-va-huong-dan-chan-doan-giam-dinh-muc-suy-giam-kha-nang-lao-dong-do-benh-nghe-nghiep--187267?tabs=tai-ve</t>
         </is>
       </c>
-      <c r="G55" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H55" s="11" t="inlineStr">
-        <is>
-          <t>Thông tư của Bộ Y tế (cần đối chiếu đúng nội dung BHXH trong danh sách)</t>
+      <c r="G55" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H55" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J55" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3280,12 +3784,24 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2019/12/45.signed.pdf</t>
         </is>
       </c>
-      <c r="G56" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H56" s="11" t="n"/>
+      <c r="G56" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H56" s="13" t="n">
+        <v>83</v>
+      </c>
+      <c r="I56" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J56" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
@@ -3316,12 +3832,24 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2015/07/84.signed.pdf</t>
         </is>
       </c>
-      <c r="G57" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H57" s="11" t="n"/>
+      <c r="G57" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H57" s="13" t="n">
+        <v>59</v>
+      </c>
+      <c r="I57" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J57" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -3352,12 +3880,24 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/7/74qh15.signed.pdf</t>
         </is>
       </c>
-      <c r="G58" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H58" s="11" t="n"/>
+      <c r="G58" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H58" s="13" t="n">
+        <v>26</v>
+      </c>
+      <c r="I58" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J58" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
@@ -3388,12 +3928,24 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/01/luat50.pdf</t>
         </is>
       </c>
-      <c r="G59" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H59" s="11" t="n"/>
+      <c r="G59" s="13" t="inlineStr">
+        <is>
+          <t>PDF có chữ (Công báo)</t>
+        </is>
+      </c>
+      <c r="H59" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="I59" s="13" t="inlineStr">
+        <is>
+          <t>Đọc lớp chữ</t>
+        </is>
+      </c>
+      <c r="J59" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="33.6" customHeight="1">
       <c r="A60" s="3" t="n">
@@ -3424,14 +3976,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2020/12/145.signed.pdf</t>
         </is>
       </c>
-      <c r="G60" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H60" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định hướng dẫn Bộ luật Lao động về điều kiện lao động và quan hệ lao động</t>
+      <c r="G60" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H60" s="13" t="n">
+        <v>122</v>
+      </c>
+      <c r="I60" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J60" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3464,14 +4024,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2020/07/88.signed.pdf</t>
         </is>
       </c>
-      <c r="G61" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H61" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định về bảo hiểm tai nạn lao động, bệnh nghề nghiệp bắt buộc</t>
+      <c r="G61" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H61" s="13" t="n">
+        <v>60</v>
+      </c>
+      <c r="I61" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J61" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3504,14 +4072,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2016/06/39.signed.pdf</t>
         </is>
       </c>
-      <c r="G62" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H62" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định hướng dẫn Luật An toàn, vệ sinh lao động</t>
+      <c r="G62" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H62" s="13" t="n">
+        <v>84</v>
+      </c>
+      <c r="I62" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J62" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3544,14 +4120,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/8/219-cp.signed.pdf</t>
         </is>
       </c>
-      <c r="G63" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H63" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định về người lao động nước ngoài làm việc tại Việt Nam</t>
+      <c r="G63" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H63" s="13" t="n">
+        <v>34</v>
+      </c>
+      <c r="I63" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J63" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3584,14 +4168,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/11/293-cp.signed.pdf</t>
         </is>
       </c>
-      <c r="G64" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H64" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định quy định mức lương tối thiểu với người lao động theo hợp đồng</t>
+      <c r="G64" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H64" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="I64" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J64" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3624,14 +4216,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/12/337-cp.signed.pdf</t>
         </is>
       </c>
-      <c r="G65" s="11" t="inlineStr">
+      <c r="G65" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H65" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="I65" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J65" s="11" t="inlineStr">
         <is>
           <t>Đã tải lại bản chính thức (file cũ của Long bị nhầm thành file đề bài)</t>
-        </is>
-      </c>
-      <c r="H65" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định (cần đối chiếu trích yếu)</t>
         </is>
       </c>
     </row>
@@ -3664,14 +4264,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2025/12/338-ndcp.signed.pdf</t>
         </is>
       </c>
-      <c r="G66" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H66" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định (cần đối chiếu trích yếu)</t>
+      <c r="G66" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H66" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="I66" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J66" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3704,14 +4312,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/01/352-nd.signed.pdf</t>
         </is>
       </c>
-      <c r="G67" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H67" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định (cần đối chiếu trích yếu)</t>
+      <c r="G67" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H67" s="13" t="n">
+        <v>55</v>
+      </c>
+      <c r="I67" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J67" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3744,14 +4360,22 @@
           <t>https://datafiles.chinhphu.vn/cpp/files/vbpq/2026/01/374-1.signed.pdf</t>
         </is>
       </c>
-      <c r="G68" s="11" t="inlineStr">
-        <is>
-          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
-        </is>
-      </c>
-      <c r="H68" s="11" t="inlineStr">
-        <is>
-          <t>Nghị định hướng dẫn một số điều của Luật Việc làm về bảo hiểm thất nghiệp</t>
+      <c r="G68" s="13" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="H68" s="13" t="n">
+        <v>45</v>
+      </c>
+      <c r="I68" s="13" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+      <c r="J68" s="11" t="inlineStr">
+        <is>
+          <t>Đúng số hiệu, đúng văn bản, đủ nội dung</t>
         </is>
       </c>
     </row>
@@ -3828,4 +4452,118 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId66"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Định dạng gốc</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Số văn bản</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Cách lấy chữ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Word gốc (.doc)</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>Đọc trực tiếp</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>PDF convert từ Word</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Đọc lớp chữ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>PDF có chữ (Công báo)</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Đọc lớp chữ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>PDF scan (chụp hình)</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n">
+        <v>55</v>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>OCR (Tesseract)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Tổng</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>65</v>
+      </c>
+      <c r="C6" s="16" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Văn bản 141/2026/NĐ-CP và 152/2025/TT-BTC thuộc 2 nhóm nên danh mục có 67 dòng cho 65 văn bản.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>